<commit_message>
Add Borrego Springs USD district intelligence profile
- Full profile: 345 students, K-12, remote desert community
- Superintendent Dr. Mark Stevens identified (email not published)
- 5 board members from Ballotpedia (3 newly elected Nov 2024)
- Board meetings indexed via Simbli eBoard (7 meetings in 2025)
- Anza-Borrego Foundation partnership: Camp Borrego, field trips, teacher PD
- CRITICAL: 15% math proficiency (vs 35% state avg) - highest need in pipeline
- Entry strategy targeting Dr. Stevens via phone (no email published)
- Budget pathway: LCFF Supp/Conc + Title I ($5-10K district-wide)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:Q4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -713,6 +713,87 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Borrego Springs USD</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>345</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>K-12</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Dr. Mark Stevens</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>29546</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>$10.5M</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>~16.8:1</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>87.2%</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>0.8%</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>8.9%</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>0.6%</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>56.7%</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -725,7 +806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -926,6 +1007,66 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Borrego Springs USD</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Agri/Tourism/Renewables</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Est. $1.5-2M</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Est. $300-500K</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Est. $10-15K</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Robotics, desert ecology, CTE pathways</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -938,7 +1079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1447,6 +1588,51 @@
       </c>
       <c r="I11" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Borrego Springs USD</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Dr. Mark Stevens</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Superintendent</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>(760) 767-5357</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>All decisions</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1540,7 +1726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2165,6 +2351,96 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Borrego Springs USD</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Anza-Borrego Foundation</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Environmental Ed</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Field trips, Camp Borrego, teacher PD</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Deep</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Key intro path for ModelIt</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Borrego Springs USD</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Simbli/eBoard</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Board management</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2177,7 +2453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2567,6 +2843,147 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Borrego Springs USD</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>K-5</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>[NEEDS VERIFICATION]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Borrego Springs USD</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>[NEEDS VERIFICATION]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Borrego Springs USD</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>9-12</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>CTE pathways active</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2579,7 +2996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2750,6 +3167,58 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Borrego Springs USD</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Dr. Mark Stevens</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Desert ecology + 15% math crisis + bilingual</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>LCFF Supp/Conc + Title I</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>$5-10K district-wide</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Mar-Jun 2026</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Phone call to superintendent</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Remote location, single decision maker, highest need district</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2762,7 +3231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2957,6 +3426,64 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Borrego Springs USD</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Dr. Mark Stevens</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Research complete</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Phone call to superintendent</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J4" t="n">
+        <v>15000</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Highest math gap in pipeline, remote but well-funded</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Fontana USD district intelligence profile
- Full profile: 33,039 students, 44 schools, K-12, San Bernardino County
- 8 contacts identified (Bergen, Lawe, Hollister, Alvarez warm, Inbody, Holley, Alegre, MacKinney)
- Board meetings indexed (2025-2026) with BoardDocs portal
- Science curriculum mapped: Discovery Ed STEM Connect + Math Techbook, Bio Animakerspace, 22 CTE pathways
- 11 vendors/partners with competitive analysis (Discovery Ed, Garner Holt, Dell 1:1, etc.)
- Entry strategy targeting Dolly Bergen (STEAM Coordinator) with Dr. Alvarez warm intro
- Budget pathway: $132M LCFF Supp/Conc + $408M Measure I Bond + CTE grants
- 3 personalized email templates, 8 talking points, 8 objection responses
- Pipeline updated (9 districts, $103-540K total estimated value)
- comparison.xlsx updated across all 8 sheets

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:Q10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1163,13 +1163,11 @@
           <t>63%</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>20.6%</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
           <t>43.8%</t>
@@ -1188,6 +1186,87 @@
       <c r="Q9" t="inlineStr">
         <is>
           <t>Rural; Math 18%, ELA 29%, Sci 19%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>San Bernardino</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>33039</v>
+      </c>
+      <c r="D10" t="n">
+        <v>44</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>K-12</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Miki R. Inbody</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>16500</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>$720M</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>24:1</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>86.5%</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>5.1%</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2.0%</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>1.0%</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>83.1%</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>24.9%</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>92.5%</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Large urban; Math 22.66%, ELA 37.35%, Sci 18.66%</t>
         </is>
       </c>
     </row>
@@ -1203,7 +1282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1770,6 +1849,68 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Est. $5-10M+</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TBD (Discovery Ed supplemental)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>i-Ready + Discovery Ed Math Techbook</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Dell 1:1 + MS365</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>NGSS + CTE PD</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>CTEIG/Perkins/SWP (22 pathways)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>$132,211,729</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Est. $15-20M</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>22 across 11 sectors</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Discovery Ed STEM Connect, Bio Animakerspace, Innovation Empire, WRO Robotics, Engineering for Kids, AVID, Dual Language Immersion</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1782,7 +1923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3124,7 +3265,6 @@
           <t>hailwood.ma@vcpusd.org</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>Administration</t>
@@ -3165,7 +3305,6 @@
           <t>clymer.ni@vcpusd.org</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>Site Admin</t>
@@ -3206,7 +3345,6 @@
           <t>rogers.aa@vcpusd.org</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>Human Resources</t>
@@ -3247,7 +3385,6 @@
           <t>howard.do@vcpusd.org</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>Student Services</t>
@@ -3283,8 +3420,6 @@
           <t>Ed Services Director</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>Education Services</t>
@@ -3302,6 +3437,366 @@
       </c>
       <c r="I34" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Dolly Bergen</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>STEAM &amp; K-12 Science Coordinator</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>dolly.bergen@fusd.net [INFERRED]</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>(909) 350-6800 x29176</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Teaching &amp; Learning</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>STEM curriculum evaluator</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Yes - STEAM lead</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Kim Lawe, Ed.D.</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Sr. Director, Career Readiness &amp; Workforce Dev.</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>kim.lawe@fusd.net [INFERRED]</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>(909) 357-5000 x29180</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>CTE / College &amp; Career</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>CTE budget authority</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Yes - CTE lead</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Christopher Hollister, Ed.D.</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Interim Assoc. Supt., Teaching &amp; Learning</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Teaching &amp; Learning</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Curriculum authority (INTERIM)</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Dr. Alejandro Alvarez (WARM)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Superintendent, Rialto USD</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>TBD (Rialto USD)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>External - Warm Connection</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Warm intro to Fontana leadership</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Yes - former Fontana career</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Miki R. Inbody</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Superintendent</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>miki.inbody@fusd.net [INFERRED]</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>(909) 357-5000</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Office of the Superintendent</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Final authority</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Danielle Holley</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Board Member, Area 4</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>danielle.holley@fusd.net</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>(909) 357-5000</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Board of Education</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Board champion potential</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Yes - former teacher, MA in C&amp;I</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Glenn Alegre</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Chief Technology Officer</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>glenn.alegre@fusd.net [INFERRED]</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Technology Services</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Tech platform approvals</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>TBD - former math teacher</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Kimberly MacKinney, Ed.D.</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Exec. Director, Secondary Schools (6-12)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Secondary Education</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>MS/HS math intervention decisions</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -3395,7 +3890,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5254,6 +5749,523 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Discovery Education</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Curriculum Publisher</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>STEM Connect (supplemental K-8) + Math Techbook (6-8)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Multi-year (since 2015)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Deep - 10+ year partnership</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>5 Moonshot elementary schools + all MS math</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Microsoft 365, Teams, Outlook, OneDrive</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>District-wide</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Vendor contract</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Primary collaboration platform</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>1:1 Latitude laptops K-12</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Since 2021-22</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Hardware vendor</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Every student has a Dell laptop</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Aeries Software</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Student Information System (SIS)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Vendor contract</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Attendance, grades, schedules</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Curriculum Associates</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>i-Ready (Math/Reading diagnostic)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Vendor contract</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>District-wide diagnostic assessment</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>NWEA</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>MAP Growth (interim assessment)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Vendor contract</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Progress monitoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Garner Holt Education</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CTE/Industry</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Bio Animakerspace at Fontana HS</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Since 2022</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Deep partnership</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>World's first bio-animatronics/neuroprosthetics lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Engineering for Kids</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>After-school STEM</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Robotics curriculum at 8 elem schools</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Program partner</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>After-school only; Upland CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>OpenGov</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>eProcurement platform</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Vendor contract</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Digital purchasing/bidding</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Chaffey College</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Higher Ed</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Dual enrollment (Automotive, general ed)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Academic partner</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>High School Partnership program</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>CSUSB</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Higher Ed</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Resident Teacher program (20 candidates)</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Academic partner</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Tuition assistance at 5 schools</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5266,7 +6278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6455,6 +7467,241 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>K-5</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Discovery Ed STEM Connect (supplemental)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Digital/Supplemental</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>5 Moonshot schools only; core science publisher TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Discovery Ed Math Techbook</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Digital/Core supplement</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>All 6th-8th grade math; core science publisher TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>9-12</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Bio-Animatronics (Garner Holt)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>CTE/Applied Science</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>World's first Bio Animakerspace at Fontana HS</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>9-12 CTE</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>22 CTE Pathways (11 sectors)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>CTE</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Various</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Various</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>CTEIG/Perkins/SWP</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Varies</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Engineering, Biotech, Mechatronics, Aviation, Fire Tech, Health Sci, Welding</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>K-12 Supplemental</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Innovation Empire Makerspace + WRO Robotics</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>STEM/Supplemental</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Various</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Measure I bond</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Stratasys 3D printers, CNC, laser cutters; WRO national/international competitors</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6467,7 +7714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6950,6 +8197,58 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Dolly Bergen (STEAM Coordinator)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>77% not meeting math + world-class STEM hardware needs modeling software + $408M Measure I + bilingual for 86% Hispanic</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>LCFF Supp/Conc ($132M) + Measure I Bond + CTE Grants + Title I</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>$40-75K pilot</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Feb-Jun 2026 LCAP cycle</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Contact Dr. Alvarez for warm intro; email Bergen + Lawe</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Feb-Mar 2026</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Large urban K-12; 33K students; Bio Animakerspace, WRO robotics, Innovation Empire; Oak Grove Prep opening Aug 2026; warm connection Dr. Alvarez (Rialto USD Supt)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6962,7 +8261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7505,6 +8804,64 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Fontana USD</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Dolly Bergen</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>dolly.bergen@fusd.net [INFERRED]</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Research complete</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Contact Dr. Alvarez for warm intro; email Bergen + Lawe</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>57500</v>
+      </c>
+      <c r="J10" t="n">
+        <v>225000</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>$40-75K pilot -&gt; $150-300K+ scale; 33K students, 77% not meeting math, $408M Measure I, Bio Animakerspace, WRO, warm connection Dr. Alvarez</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Brawley Elementary SD district intelligence profile
- Full profile: 3,883 students TK-8, Imperial County, CDS 13-63073-0000000
- 26 contacts identified across 6 tiers with verified email pattern (finitial.last@besd.org)
- Board meetings indexed (2025-present) via AgendaOnline
- Science curriculum white space confirmed — NO publisher identified (primary entry point)
- CAST science: 12.93% overall, 1.61% EL (bilingual platform unique differentiator)
- Math decline: 32% Grade 3 → 12% Grade 8 (highest-impact pitch data)
- Padilla-Pace MS (opened Aug 2024) identified as greenfield pilot site
- New superintendent Luis Panduro: former Dir. Instructional Technology + Asst. Supt. Curriculum
- Budget pathway: Title IV-A + LCFF Supplemental + GEAR UP/Project R.I.S.E.
- Entry targeting Victor Ramirez (Dir. Technology) + Lynn Lizarraga (Math Dept Head)
- Pipeline: Stage 1 (16 total districts now), est. value $5-10K pilot → $25-50K scale

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1519,6 +1519,87 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Brawley Elementary SD</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Imperial</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>3883</v>
+      </c>
+      <c r="D14" t="n">
+        <v>10</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>TK-8</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Luis Panduro</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>14548</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>~$69.9M</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>95.0%</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>0.8%</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>3.3%</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>~84.6%</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>~39.3%</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>N/A (TK-8)</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1531,7 +1612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2326,6 +2407,66 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Brawley Elementary SD</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>TBD (white space)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>McGraw-Hill Connected</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>PowerSchool + Achieve3000 + Renaissance STAR</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>N/A (TK-8)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>TBD (est. via LCFF Supp/Conc + Title IV-A)</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>TBD (Title IV-A eligible)</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Smart Start Saturdays (STEAM), Camp Adventure Intersession, ASES After-School, GEAR UP/R.I.S.E., Dual Language Immersion</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2338,7 +2479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4909,6 +5050,96 @@
         <v>5</v>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Brawley Elementary SD</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Victor Ramirez</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Director of Technology</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>vramirez@besd.org</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>EdTech platform approval; primary decision maker</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Brawley Elementary SD</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Lynn Lizarraga</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Dept. Head Mathematics</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>llizarraga@besd.org</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Mathematics / Curriculum</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Math curriculum &amp; intervention decisions; STEM champion</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4921,7 +5152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4988,6 +5219,58 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Brawley Elementary SD</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TBD - Padilla-Pace MS greenfield build</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Facilities / New School</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>New middle school greenfield; key entry point for ModelIt pilot</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5000,7 +5283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8783,6 +9066,335 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Brawley Elementary SD</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>McGraw-Hill Connected</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Math curriculum TK-8</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Annual contract</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Primary math curriculum</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Brawley Elementary SD</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Achieve3000</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>EdTech</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Differentiated reading/ELA platform</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Annual contract</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>EL literacy support</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Brawley Elementary SD</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Renaissance Learning (STAR)</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Math + reading diagnostic screener</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>No - different use</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Annual contract</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Universal screener</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Brawley Elementary SD</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>PowerSchool</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Student Information System (SIS)</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Annual contract</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Primary SIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Brawley Elementary SD</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>ICOE</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Regional Agency</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Imperial County Office of Education - instructional support</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Institutional</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>County-level support and PD</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Brawley Elementary SD</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>SDSU-IV (GEAR UP)</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Higher Ed / Federal Grant</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>GEAR UP / R.I.S.E. college-readiness program</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Federal grant</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Grant partner</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Targets low-income students for college readiness</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Brawley Elementary SD</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Imperial Valley College</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Higher Ed</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Dual enrollment pipeline / college readiness</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Community partnership</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Local community college partner</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8795,7 +9407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10783,6 +11395,53 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Brawley Elementary SD</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>TK-8</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Unknown / TBD</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Science curriculum not publicly confirmed (white space); significant ModelIt opportunity</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10795,7 +11454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11476,6 +12135,58 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Brawley Elementary SD</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Victor Ramirez, Dir. of Technology (vramirez@besd.org)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1.61% EL science proficiency + new Padilla-Pace MS greenfield + bilingual platform for 95% Hispanic, 39% EL district</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Title IV-A + LCFF Supplemental</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>$5-10K pilot → $25-50K scale</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Mar-Jun 2026 (LCAP window)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Send intro email to Ramirez + Lizarraga + Vildosola</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>95% Hispanic, 39.3% EL, 84.6% ED; 1.61% EL science proficiency is lowest viable entry hook; greenfield MS is greenfield opportunity; priority score 95/100</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11488,7 +12199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12251,6 +12962,64 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Brawley Elementary SD</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Victor Ramirez</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>vramirez@besd.org</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Research complete</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Send intro email to Ramirez + Lizarraga + Vildosola</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>7500</v>
+      </c>
+      <c r="J14" t="n">
+        <v>37500</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>95/100 priority; 95% Hispanic, 39.3% EL, 1.61% EL science proficiency; greenfield Padilla-Pace MS; science curriculum white space; Imperial Valley isolation = low competition</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Calexico USD district intelligence profile
- Full profile with demographics (99.1% Hispanic), CAST scores (12.87% science, 60% Nearly Met), and STEM programs
- 25+ contacts identified including Korina Tabarez (Academics & Instruction), both Jr. High principals, and full board
- Board meetings indexed (2025-present) with purchasing/warrants extraction template
- Science curriculum: GREENFIELD — no confirmed vendor; major opportunity
- 7 vendors/partners mapped (Synergy, Naviance, Google, Afterschool Unlimited)
- Entry strategy targeting Korina Tabarez + SPARKs after-school entry via Esmeralda Garcia
- Budget pathway: Title IV-A + LCFF Supplemental/Concentration
- Hook: 12.87% CAST science, 60% Nearly Met cohort, Measure Q $47M STEM buildings, bilingual border community
- CDE priority score: 95/100

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1600,6 +1600,87 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Imperial</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>8351</v>
+      </c>
+      <c r="D15" t="n">
+        <v>12</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>K-12</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Arturo Jimenez</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>19484</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>$185.87M</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>22.84:1</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>99.1%</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>0.4%</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>0.2%</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>56.8%</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>8.8%</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>87-93%</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1612,7 +1693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2467,6 +2548,66 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>TBD (no confirmed vendor)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>TBD (1:1 devices in progress)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Est. $500K+ (10 CTE pathways)</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Est. large (56.8% SED)</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Active (multiple schools)</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Est. $150-200K</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>10</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>SPARKs (STEM after-school), Lego Education, Unimatics Robotics (historical), AVID, NJROTC, Measure Q STEM buildings (CHS)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2479,7 +2620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5138,6 +5279,241 @@
       </c>
       <c r="I59" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Korina Tabarez</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Coordinator, Academics &amp; Instruction</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>ktabarez@cusdk12.org</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>(760) 768-3888</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Educational Services</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Curriculum adoption decisions; closest contact to science curriculum selection</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Tier 1 — Primary</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Esmeralda Garcia</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Director, Expanded Learning (SPARKs)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>egarcia@cusdk12.org</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>(760) 768-3888</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Expanded Learning</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>After-school STEM programming; independent ASES budget</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Tier 1 — After-School Entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Elisa Ramirez</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Asst. Superintendent, Educational Services</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>eramirez@cusdk12.org</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>(760) 768-3892</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Educational Services</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Curriculum authority; approves major program partnerships</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Diego Romero</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Principal, Enrique Camarena Jr. High</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>dromero@cusdk12.org</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>(760) 768-3808 ext. 6599</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Camarena Jr. High</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Primary pilot school principal; Grade 8 CAST target</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Tier 4 — Pilot School</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Arturo Jimenez</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Superintendent</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>ajimenez@cusdk12.org</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>(760) 768-3888</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Superintendent Office</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Final approval authority; bilingual/equity champion</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -5283,7 +5659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I89"/>
+  <dimension ref="A1:I97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9395,6 +9771,382 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Edupoint Synergy</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Student Information System (SIS)</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Deep</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Confirmed - core infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Naviance</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>College planning / career exploration (CHS)</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Confirmed at Calexico High School</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Productivity, LMS (Classroom), Chromebooks</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Deep</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Confirmed - district standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Afterschool Unlimited</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Community Partner</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>SPARKs after-school operator ($1.2M contract)</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>$1.2M/yr</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>2025-26+</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Confirmed - Aug. 2025 board renewal</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Imperial Valley College</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Higher Ed Partner</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Dual enrollment</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Located in El Centro; provides dual enrollment for CHS</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>SDSU Imperial Valley</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Higher Ed Partner</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>University partner in Calexico</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Low-Medium</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Campus located in Calexico</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Calexico Educational Foundation</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Community/Foundation</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Grants, robotics team (Unimatics) funding</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>alimon@cusdk12.org - Foundation Director Alejandra Limon</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Science Curriculum (UNKNOWN)</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Curriculum Publisher</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>K-12 science curriculum - NOT CONFIRMED</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>No confirmed vendor - GREENFIELD OPPORTUNITY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9407,7 +10159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11442,6 +12194,147 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>K-6 (Elementary)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>NOT CONFIRMED</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>No confirmed publisher; CAST Gr. 5 = 10.94% — greenfield for ModelIt</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>7-8 (Junior High)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>NOT CONFIRMED</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>CAST Gr. 8 = 14.09%; 58% Nearly Met; top pilot target grade band</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>9-12 (High School)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>NOT CONFIRMED + Naviance</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Unknown + College Planning</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>CAST Gr. 11 = 13.49%; 65.73% Nearly Met — highest Nearly Met of all grades; Measure Q STEM buildings opening</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11454,7 +12347,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12187,6 +13080,58 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Korina Tabarez (Coordinator, Academics &amp; Instruction)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>12.87% CAST science; 60% Nearly Met at every grade; no confirmed science curriculum vendor; $47M Measure Q STEM buildings; bilingual border community (99% Hispanic)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Title IV-A + LCFF Supplemental/Concentration</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>$8-15K pilot / $75-120K district-wide</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Mar-Jun 2026 (LCAP cycle)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Send intro email — CAST Nearly Met hook + bilingual + Measure Q STEM</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Greenfield district (no science vendor); SPARKs after-school pilot entry; Supt. is bilingual equity champion</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12199,7 +13144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13020,6 +13965,64 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Calexico USD</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Korina Tabarez</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>ktabarez@cusdk12.org</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Research complete</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Send intro email — 12.87% CAST science + Nearly Met + bilingual + Measure Q STEM hook</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J15" t="n">
+        <v>100000</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>99% Hispanic, 12.87% science, greenfield curriculum, Measure Q STEM buildings, bilingual platform fit, CDE priority 95/100</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Panama-Buena Vista Union district intelligence profile
- Full profile: 19,366 students, 26 campuses (19 elem + 5 JH + 2 TK-8), Kern County
- 35+ contacts identified with verified emails (pattern: finitial+lastname@pbvusd.k12.ca.us)
- Primary contact: Dr. Valerie Park, Director ACT (vpark@pbvusd.k12.ca.us, ext. 6349)
- Board meetings indexed (2025, Simbli eBoard system)
- Science curriculum: OPEN WHITE SPACE — no confirmed incumbent publisher K-8
- Key vendors mapped: Canvas, ClassLink, Synergy, McGraw Hill/HMH (math+ELA), Renaissance
- Entry strategy targeting Dir. ACT + 5 JH principals as pilot sites
- Budget pathway: LCFF Supplemental/Concentration (62% Hispanic + 14.5% EL)
- CAST science 26.45% overall; EL science 7.48% — bilingual platform directly relevant
- Priority score: 95/100 | Est. deal: $50-100K district-wide

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1829,6 +1829,73 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Panama-Buena Vista Union School District</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Kern</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>19366</v>
+      </c>
+      <c r="D18" t="n">
+        <v>26</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>TK-8</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Dr. Katie Russell</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>13924</v>
+      </c>
+      <c r="H18" t="n">
+        <v>338300000</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>62.1</v>
+      </c>
+      <c r="K18" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="L18" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="M18" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="N18" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="O18" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>N/A - TK-8 district</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>95/100 CDE Priority</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1841,7 +1908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2878,6 +2945,66 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Panama-Buena Vista Union School District</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TBD (est. $200-400K)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>TBD - no confirmed publisher (greenfield)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>N/A - TK-8 district</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>TBD - est. significant LCFF Supp/Conc from $338.3M total revenue</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2890,7 +3017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6246,6 +6373,53 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Panama-Buena Vista Union School District</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Dr. Valerie Park</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Director, ACT</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>vpark@pbvusd.k12.ca.us</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Academics/Curriculum</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Primary decision-maker for curriculum adoption</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>1 - Primary</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6258,7 +6432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6481,6 +6655,58 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Panama-Buena Vista Union School District</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TBD - review needed</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Science curriculum adoption (est.)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>LCFF Supplemental/Concentration</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Unknown - no confirmed science publisher</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>No confirmed science curriculum vendor; greenfield opportunity; 26.45% CAST science</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6493,7 +6719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I110"/>
+  <dimension ref="A1:I117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11592,6 +11818,335 @@
         </is>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Panama-Buena Vista Union School District</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Canvas</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Technology - LMS</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Learning Management System</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>LMS in use</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Panama-Buena Vista Union School District</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>ClassLink</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Technology - SSO</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Single Sign-On</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>SSO platform</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Panama-Buena Vista Union School District</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Synergy</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Technology - SIS</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Student Information System</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>SIS in use</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Panama-Buena Vista Union School District</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>McGraw Hill/HMH</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Curriculum - Math/ELA</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Math and ELA instruction</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Math + ELA publisher; confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Panama-Buena Vista Union School District</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Renaissance Learning</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Reading/math assessment and intervention</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Confirmed vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Panama-Buena Vista Union School District</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>ELLevation</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>EL Support</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>English Language Learner support platform</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>EL platform; 14.5% EL population</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Panama-Buena Vista Union School District</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Science Curriculum (UNKNOWN)</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Curriculum - Science</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>K-8 science instruction</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>No confirmed science publisher — greenfield opportunity</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11604,7 +12159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14062,6 +14617,100 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Panama-Buena Vista Union School District</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>K-5</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Unknown (TBD)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>No confirmed publisher — complete white space</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Panama-Buena Vista Union School District</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Unknown (TBD)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>No confirmed publisher — complete white space; 26.45% CAST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14074,7 +14723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14963,6 +15612,58 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Panama-Buena Vista Union School District</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Dr. Valerie Park, Director ACT (vpark@pbvusd.k12.ca.us)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>43% math Grade 3 drops to 22% Grade 8; 7.48% EL science CAST; no confirmed science publisher; 19K students = major scale opportunity</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>LCFF Supplemental/Concentration</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>$50-100K district-wide</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>March 2026 outreach → May-June 2026 pilot → June 2026 LCAP inclusion → Sep 2026 paid contract</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Email Dr. Valerie Park + IS Coordinators (Wave 1)</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>March 2026</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Greenfield science publisher; 19,366 students; 26 schools; 30.2% math; 26.45% science; 62.1% Hispanic; 14.5% EL; 14.3% SED (likely understated); Canvas+ClassLink+Synergy in place; CDE priority 95/100</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14975,7 +15676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15974,6 +16675,68 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Panama-Buena Vista Union School District</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Dr. Valerie Park</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>vpark@pbvusd.k12.ca.us</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Research complete; profile built</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Send intro email to Dr. Valerie Park + IS Coordinators</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>March 2026</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>TBD (est. $20-40K pilot)</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>$50-100K district-wide</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Medium-High</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Greenfield science publisher; 19K students; 26 schools; 30.2% math; 26.45% science; 43% math Gr3 drops to 22% Gr8; Canvas+ClassLink+Synergy deployed; no confirmed science vendor; 95/100 CDE priority</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>